<commit_message>
Add economic impact and Fed action columns, use official data sources
- Add shared utility module (scripts/utils/excel-writer.js) with automatic
  computation of Economic Impact and Expected Fed Action based on thresholds
- Update all indicator scripts to use official data sources:
  - BLS for unemployment, nonfarm payrolls, CPI, PPI
  - ISM press releases via PR Newswire for manufacturing/services PMI
  - Conference Board for consumer confidence
  - DOL PDF for jobless claims
- Add collect:all npm script for single-command data collection
- Update README with Quick Start section
- Chicago PMI requires MNI subscription (manual entry documented)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/macro-indicators.xlsx
+++ b/data/macro-indicators.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
   <si>
     <t>Indicator</t>
   </si>
@@ -19,34 +19,91 @@
     <t>Value</t>
   </si>
   <si>
+    <t>Economic Impact</t>
+  </si>
+  <si>
+    <t>Expected Fed Action</t>
+  </si>
+  <si>
     <t>Last Updated</t>
   </si>
   <si>
+    <t>CPI YoY</t>
+  </si>
+  <si>
+    <t>2.7%</t>
+  </si>
+  <si>
+    <t>High inflation</t>
+  </si>
+  <si>
+    <t>Contractionary</t>
+  </si>
+  <si>
+    <t>1/27/2026, 10:38:55 PM</t>
+  </si>
+  <si>
+    <t>Core CPI YoY</t>
+  </si>
+  <si>
+    <t>0.2%</t>
+  </si>
+  <si>
+    <t>Low inflation</t>
+  </si>
+  <si>
+    <t>Expansionary</t>
+  </si>
+  <si>
+    <t>ISM Manufacturing PMI</t>
+  </si>
+  <si>
+    <t>Contraction</t>
+  </si>
+  <si>
+    <t>1/27/2026, 10:39:07 PM</t>
+  </si>
+  <si>
+    <t>Consumer Confidence</t>
+  </si>
+  <si>
+    <t>Negative sentiment</t>
+  </si>
+  <si>
+    <t>1/27/2026, 10:39:22 PM</t>
+  </si>
+  <si>
+    <t>PPI MoM</t>
+  </si>
+  <si>
+    <t>+0.2%</t>
+  </si>
+  <si>
+    <t>1/27/2026, 10:39:32 PM</t>
+  </si>
+  <si>
+    <t>ISM Non-Manufacturing PMI</t>
+  </si>
+  <si>
+    <t>OK expansion</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>1/27/2026, 10:39:44 PM</t>
+  </si>
+  <si>
     <t>Unemployment Rate</t>
   </si>
   <si>
-    <t>1/27/2026, 9:28:11 PM</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Week 1</t>
-  </si>
-  <si>
-    <t>Week 2</t>
-  </si>
-  <si>
-    <t>Week 3</t>
-  </si>
-  <si>
-    <t>Week 4</t>
-  </si>
-  <si>
-    <t>Week 5</t>
-  </si>
-  <si>
-    <t>Initial Jobless Claims</t>
+    <t>4.4%</t>
+  </si>
+  <si>
+    <t>OK economy</t>
+  </si>
+  <si>
+    <t>1/27/2026, 10:41:18 PM</t>
   </si>
   <si>
     <t>Nonfarm Payrolls</t>
@@ -55,7 +112,10 @@
     <t>+50,000</t>
   </si>
   <si>
-    <t>1/27/2026, 9:35:32 PM</t>
+    <t>Strong economy</t>
+  </si>
+  <si>
+    <t>1/27/2026, 10:41:23 PM</t>
   </si>
 </sst>
 </file>
@@ -94,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -102,7 +162,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -442,15 +501,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="3" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -460,67 +520,147 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2">
-        <v>4.4</v>
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="1" t="s">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
+        <v>14</v>
+      </c>
+      <c r="B4" s="2">
+        <v>47.9</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="2">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="2">
+        <v>89.1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>14</v>
+      <c r="E5" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="2">
+        <v>54.4</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Switch BLS scrapers to public API to fix bot detection blocks
BLS website now blocks Playwright-based scraping. Replaced all four
BLS scripts (unemployment rate, nonfarm payrolls, CPI/Core CPI, PPI)
with direct BLS Public API calls, eliminating the Playwright dependency
for these indicators.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/macro-indicators.xlsx
+++ b/data/macro-indicators.xlsx
@@ -5,13 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="January 2026" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="February 2026" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="March 2026" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="64">
   <si>
     <t>Indicator</t>
   </si>
@@ -40,28 +42,28 @@
     <t>Contractionary</t>
   </si>
   <si>
-    <t>1/27/2026, 10:38:55 PM</t>
+    <t>1/28/2026, 9:23:19 PM</t>
   </si>
   <si>
     <t>Core CPI YoY</t>
   </si>
   <si>
-    <t>0.2%</t>
-  </si>
-  <si>
-    <t>Low inflation</t>
+    <t>2.6%</t>
+  </si>
+  <si>
+    <t>1/28/2026, 9:23:26 PM</t>
+  </si>
+  <si>
+    <t>ISM Manufacturing PMI</t>
+  </si>
+  <si>
+    <t>Contraction</t>
   </si>
   <si>
     <t>Expansionary</t>
   </si>
   <si>
-    <t>ISM Manufacturing PMI</t>
-  </si>
-  <si>
-    <t>Contraction</t>
-  </si>
-  <si>
-    <t>1/27/2026, 10:39:07 PM</t>
+    <t>1/27/2026, 10:44:37 PM</t>
   </si>
   <si>
     <t>Consumer Confidence</t>
@@ -70,7 +72,7 @@
     <t>Negative sentiment</t>
   </si>
   <si>
-    <t>1/27/2026, 10:39:22 PM</t>
+    <t>1/27/2026, 10:45:00 PM</t>
   </si>
   <si>
     <t>PPI MoM</t>
@@ -79,7 +81,7 @@
     <t>+0.2%</t>
   </si>
   <si>
-    <t>1/27/2026, 10:39:32 PM</t>
+    <t>1/27/2026, 10:44:26 PM</t>
   </si>
   <si>
     <t>ISM Non-Manufacturing PMI</t>
@@ -91,7 +93,7 @@
     <t>Neutral</t>
   </si>
   <si>
-    <t>1/27/2026, 10:39:44 PM</t>
+    <t>1/27/2026, 10:44:46 PM</t>
   </si>
   <si>
     <t>Unemployment Rate</t>
@@ -103,7 +105,7 @@
     <t>OK economy</t>
   </si>
   <si>
-    <t>1/27/2026, 10:41:18 PM</t>
+    <t>1/27/2026, 10:44:11 PM</t>
   </si>
   <si>
     <t>Nonfarm Payrolls</t>
@@ -115,7 +117,94 @@
     <t>Strong economy</t>
   </si>
   <si>
-    <t>1/27/2026, 10:41:23 PM</t>
+    <t>1/27/2026, 10:44:16 PM</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Initial Jobless Claims</t>
+  </si>
+  <si>
+    <t>05/02/2026, 2:11:52 am</t>
+  </si>
+  <si>
+    <t>05/02/2026, 2:11:56 am</t>
+  </si>
+  <si>
+    <t>05/02/2026, 2:12:02 am</t>
+  </si>
+  <si>
+    <t>05/02/2026, 2:12:09 am</t>
+  </si>
+  <si>
+    <t>+0.5%</t>
+  </si>
+  <si>
+    <t>05/02/2026, 2:12:14 am</t>
+  </si>
+  <si>
+    <t>05/02/2026, 2:12:27 am</t>
+  </si>
+  <si>
+    <t>05/02/2026, 2:12:38 am</t>
+  </si>
+  <si>
+    <t>05/02/2026, 2:12:52 am</t>
+  </si>
+  <si>
+    <t>29/03/2026, 9:58:09 pm</t>
+  </si>
+  <si>
+    <t>Strong expansion</t>
+  </si>
+  <si>
+    <t>29/03/2026, 9:58:18 pm</t>
+  </si>
+  <si>
+    <t>29/03/2026, 9:58:32 pm</t>
+  </si>
+  <si>
+    <t>29/03/2026, 9:57:54 pm</t>
+  </si>
+  <si>
+    <t>-92,000</t>
+  </si>
+  <si>
+    <t>Weak economy</t>
+  </si>
+  <si>
+    <t>29/03/2026, 9:57:55 pm</t>
+  </si>
+  <si>
+    <t>2.4%</t>
+  </si>
+  <si>
+    <t>OK inflation</t>
+  </si>
+  <si>
+    <t>29/03/2026, 9:57:57 pm</t>
+  </si>
+  <si>
+    <t>2.5%</t>
+  </si>
+  <si>
+    <t>29/03/2026, 9:57:58 pm</t>
   </si>
 </sst>
 </file>
@@ -154,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -162,6 +251,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -501,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -552,27 +642,27 @@
         <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2">
         <v>47.9</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>16</v>
@@ -589,7 +679,7 @@
         <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>19</v>
@@ -661,6 +751,502 @@
       </c>
       <c r="E9" s="2" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11" s="2">
+        <v>200000</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="2">
+        <v>209000</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="2">
+        <v>52.6</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="2">
+        <v>53.8</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="2">
+        <v>84.5</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="2">
+        <v>210000</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2">
+        <v>52.4</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="2">
+        <v>56.1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="2">
+        <v>91.2</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>